<commit_message>
Actualización de Sprint Planner
</commit_message>
<xml_diff>
--- a/Team72_Energi_AI_Sprint_Planner.xlsx
+++ b/Team72_Energi_AI_Sprint_Planner.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Zuleyca Soto\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Desktop\Google Drive sincronizar\NoCountry Hackaton ONE\Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3C0F56B-3BC9-4DA6-837A-BB6F74ED3FAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{049E31A3-01A6-4845-BAF0-EA9B0BBC94FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Resumen y Equipo" sheetId="1" r:id="rId1"/>
     <sheet name="Cronograma de Trabajo" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Cronograma de Trabajo'!$A$6:$M$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Cronograma de Trabajo'!$A$6:$M$32</definedName>
   </definedNames>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="201">
   <si>
     <t>Generated 2026-07-16 | v1.0</t>
   </si>
@@ -66,9 +66,6 @@
     <t>Resumen y Equipo</t>
   </si>
   <si>
-    <t>Visión general, equipo de 8 personas, roles y convenciones de formato.</t>
-  </si>
-  <si>
     <t>Cronograma de Trabajo</t>
   </si>
   <si>
@@ -117,9 +114,6 @@
     <t>Despliegue de Spring Boot en OCI Compute, containerización con Docker, documentación con Swagger/OpenAPI.</t>
   </si>
   <si>
-    <t>Jesús Guadalupe Rivera Meza</t>
-  </si>
-  <si>
     <t>Data Scientist</t>
   </si>
   <si>
@@ -297,9 +291,6 @@
     <t>Simular y preparar el dataset de consumo energético (CSV)</t>
   </si>
   <si>
-    <t>Jesús (DS)</t>
-  </si>
-  <si>
     <t>OCI Object Storage</t>
   </si>
   <si>
@@ -640,6 +631,18 @@
   </si>
   <si>
     <t>Generated 2026-07-20 | v1.1</t>
+  </si>
+  <si>
+    <t>Sandra Arboleda y Zuleyca Balles</t>
+  </si>
+  <si>
+    <t>Sandra y Zuleyca (DS)</t>
+  </si>
+  <si>
+    <t>Visión general, equipo de 7 personas, roles y convenciones de formato.</t>
+  </si>
+  <si>
+    <t>Completada</t>
   </si>
 </sst>
 </file>
@@ -1147,33 +1150,34 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C29"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="25" customWidth="1"/>
+    <col min="1" max="1" width="44.7109375" customWidth="1"/>
+    <col min="2" max="2" width="25" customWidth="1"/>
     <col min="3" max="3" width="75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>4</v>
       </c>
@@ -1184,192 +1188,192 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>7</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>8</v>
+        <v>199</v>
       </c>
       <c r="C8" s="8" t="str">
         <f>HYPERLINK("#'Resumen y Equipo'!A1", "Ir a Resumen")</f>
         <v>Ir a Resumen</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="7" t="s">
         <v>9</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>10</v>
       </c>
       <c r="C9" s="8" t="str">
         <f>HYPERLINK("#'Cronograma de Trabajo'!A1", "Ir a Cronograma")</f>
         <v>Ir a Cronograma</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A13" s="5" t="s">
+      <c r="B13" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="C13" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C13" s="5" t="s">
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="6" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A14" s="6" t="s">
+      <c r="B14" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="9" t="s">
+      <c r="C14" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C14" s="7" t="s">
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="6" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A15" s="6" t="s">
+      <c r="B15" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="B15" s="9" t="s">
+      <c r="C15" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="7" t="s">
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="6" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A16" s="6" t="s">
+      <c r="B16" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C16" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B16" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="C16" s="7" t="s">
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A17" s="6" t="s">
+      <c r="B17" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C17" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B17" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="C17" s="7" t="s">
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="B18" s="9" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A18" s="6" t="s">
+      <c r="C18" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B18" s="9" t="s">
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="B19" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C19" s="7" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A19" s="6" t="s">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C19" s="7" t="s">
+      <c r="B20" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C20" s="7" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A20" s="6" t="s">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B20" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C20" s="7" t="s">
+      <c r="B21" s="9" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A21" s="6" t="s">
+      <c r="C21" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B21" s="9" t="s">
+    </row>
+    <row r="24" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="C21" s="7" t="s">
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" s="5" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="4" t="s">
+      <c r="B25" s="5" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A25" s="5" t="s">
+      <c r="C25" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="B25" s="5" t="s">
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="C25" s="5" t="s">
+      <c r="B26" s="7" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A26" s="10" t="s">
+      <c r="C26" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="B26" s="7" t="s">
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="C26" s="7" t="s">
+      <c r="B27" s="7" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A27" s="11" t="s">
+      <c r="C27" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="B27" s="7" t="s">
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="C27" s="7" t="s">
+      <c r="B28" s="7" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A28" s="12" t="s">
+      <c r="C28" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B28" s="7" t="s">
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="C28" s="7" t="s">
+      <c r="B29" s="7" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A29" s="13" t="s">
+      <c r="C29" s="7" t="s">
         <v>48</v>
-      </c>
-      <c r="B29" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="C29" s="7" t="s">
-        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -1381,98 +1385,98 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:M39"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="77" customWidth="1"/>
     <col min="2" max="2" width="11" customWidth="1"/>
     <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="45" customWidth="1"/>
-    <col min="5" max="5" width="18" customWidth="1"/>
+    <col min="4" max="4" width="64.7109375" customWidth="1"/>
+    <col min="5" max="5" width="21" customWidth="1"/>
     <col min="6" max="6" width="15" customWidth="1"/>
     <col min="7" max="7" width="21" customWidth="1"/>
     <col min="8" max="9" width="13" customWidth="1"/>
     <col min="10" max="11" width="12" customWidth="1"/>
-    <col min="12" max="12" width="25" customWidth="1"/>
-    <col min="13" max="13" width="45" customWidth="1"/>
+    <col min="12" max="12" width="29.5703125" customWidth="1"/>
+    <col min="13" max="13" width="69.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.5">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="14" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
+      <c r="B6" s="14" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="6" spans="1:13" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="14" t="s">
+      <c r="C6" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="D6" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="C6" s="14" t="s">
+      <c r="E6" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="D6" s="14" t="s">
+      <c r="F6" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="E6" s="14" t="s">
+      <c r="G6" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="F6" s="14" t="s">
+      <c r="H6" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="G6" s="14" t="s">
+      <c r="I6" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="H6" s="14" t="s">
+      <c r="J6" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="I6" s="14" t="s">
+      <c r="K6" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="J6" s="14" t="s">
+      <c r="L6" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="K6" s="14" t="s">
+      <c r="M6" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="L6" s="14" t="s">
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A7" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="M6" s="14" t="s">
+      <c r="B7" s="15" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A7" s="15" t="s">
+      <c r="C7" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="B7" s="15" t="s">
+      <c r="D7" s="16" t="s">
         <v>67</v>
       </c>
-      <c r="C7" s="16" t="s">
+      <c r="E7" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="D7" s="16" t="s">
+      <c r="F7" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="E7" s="16" t="s">
+      <c r="G7" s="15" t="s">
         <v>70</v>
-      </c>
-      <c r="F7" s="15" t="s">
-        <v>71</v>
-      </c>
-      <c r="G7" s="15" t="s">
-        <v>72</v>
       </c>
       <c r="H7" s="17">
         <v>46220</v>
@@ -1485,36 +1489,36 @@
         <v>2</v>
       </c>
       <c r="K7" s="19" t="s">
+        <v>200</v>
+      </c>
+      <c r="L7" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="M7" s="16" t="s">
         <v>73</v>
       </c>
-      <c r="L7" s="16" t="s">
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A8" s="15" t="s">
         <v>74</v>
       </c>
-      <c r="M7" s="16" t="s">
+      <c r="B8" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="C8" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="D8" s="16" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A8" s="15" t="s">
+      <c r="E8" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="F8" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="B8" s="15" t="s">
-        <v>67</v>
-      </c>
-      <c r="C8" s="16" t="s">
-        <v>68</v>
-      </c>
-      <c r="D8" s="16" t="s">
-        <v>77</v>
-      </c>
-      <c r="E8" s="16" t="s">
-        <v>70</v>
-      </c>
-      <c r="F8" s="15" t="s">
-        <v>78</v>
-      </c>
       <c r="G8" s="15" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H8" s="17">
         <v>46222</v>
@@ -1527,36 +1531,36 @@
         <v>2</v>
       </c>
       <c r="K8" s="19" t="s">
+        <v>200</v>
+      </c>
+      <c r="L8" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="M8" s="16" t="s">
         <v>79</v>
       </c>
-      <c r="L8" s="16" t="s">
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A9" s="15" t="s">
         <v>80</v>
       </c>
-      <c r="M8" s="16" t="s">
+      <c r="B9" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="C9" s="16" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A9" s="15" t="s">
+      <c r="D9" s="16" t="s">
         <v>82</v>
       </c>
-      <c r="B9" s="15" t="s">
-        <v>67</v>
-      </c>
-      <c r="C9" s="16" t="s">
-        <v>83</v>
-      </c>
-      <c r="D9" s="16" t="s">
-        <v>84</v>
-      </c>
       <c r="E9" s="16" t="s">
-        <v>85</v>
+        <v>198</v>
       </c>
       <c r="F9" s="15" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="G9" s="15" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="H9" s="17">
         <v>46220</v>
@@ -1569,36 +1573,36 @@
         <v>3</v>
       </c>
       <c r="K9" s="19" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="L9" s="16" t="s">
+        <v>83</v>
+      </c>
+      <c r="M9" s="16" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A10" s="15" t="s">
+        <v>85</v>
+      </c>
+      <c r="B10" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>81</v>
+      </c>
+      <c r="D10" s="16" t="s">
         <v>86</v>
       </c>
-      <c r="M9" s="16" t="s">
+      <c r="E10" s="16" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A10" s="15" t="s">
-        <v>88</v>
-      </c>
-      <c r="B10" s="15" t="s">
-        <v>67</v>
-      </c>
-      <c r="C10" s="16" t="s">
-        <v>83</v>
-      </c>
-      <c r="D10" s="16" t="s">
-        <v>89</v>
-      </c>
-      <c r="E10" s="16" t="s">
-        <v>90</v>
-      </c>
       <c r="F10" s="15" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G10" s="15" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="H10" s="17">
         <v>46223</v>
@@ -1611,36 +1615,36 @@
         <v>2</v>
       </c>
       <c r="K10" s="19" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="L10" s="16" t="s">
+        <v>88</v>
+      </c>
+      <c r="M10" s="16" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A11" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="B11" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="C11" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="M10" s="16" t="s">
+      <c r="D11" s="16" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A11" s="15" t="s">
+      <c r="E11" s="16" t="s">
         <v>93</v>
       </c>
-      <c r="B11" s="15" t="s">
-        <v>67</v>
-      </c>
-      <c r="C11" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="D11" s="16" t="s">
-        <v>95</v>
-      </c>
-      <c r="E11" s="16" t="s">
-        <v>96</v>
-      </c>
       <c r="F11" s="15" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="G11" s="15" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="H11" s="17">
         <v>46220</v>
@@ -1653,36 +1657,36 @@
         <v>3</v>
       </c>
       <c r="K11" s="19" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="L11" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="M11" s="16" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A12" s="15" t="s">
+        <v>96</v>
+      </c>
+      <c r="B12" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="C12" s="16" t="s">
         <v>97</v>
       </c>
-      <c r="M11" s="16" t="s">
+      <c r="D12" s="16" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A12" s="15" t="s">
+      <c r="E12" s="16" t="s">
         <v>99</v>
       </c>
-      <c r="B12" s="15" t="s">
-        <v>67</v>
-      </c>
-      <c r="C12" s="16" t="s">
-        <v>100</v>
-      </c>
-      <c r="D12" s="16" t="s">
-        <v>101</v>
-      </c>
-      <c r="E12" s="16" t="s">
-        <v>102</v>
-      </c>
       <c r="F12" s="15" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="G12" s="15" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="H12" s="17">
         <v>46220</v>
@@ -1695,36 +1699,36 @@
         <v>3</v>
       </c>
       <c r="K12" s="19" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="L12" s="16" t="s">
+        <v>100</v>
+      </c>
+      <c r="M12" s="16" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A13" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="B13" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="C13" s="16" t="s">
+        <v>97</v>
+      </c>
+      <c r="D13" s="16" t="s">
         <v>103</v>
       </c>
-      <c r="M12" s="16" t="s">
+      <c r="E13" s="16" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A13" s="15" t="s">
-        <v>105</v>
-      </c>
-      <c r="B13" s="15" t="s">
-        <v>67</v>
-      </c>
-      <c r="C13" s="16" t="s">
-        <v>100</v>
-      </c>
-      <c r="D13" s="16" t="s">
-        <v>106</v>
-      </c>
-      <c r="E13" s="16" t="s">
-        <v>107</v>
-      </c>
       <c r="F13" s="15" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G13" s="15" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="H13" s="17">
         <v>46223</v>
@@ -1737,36 +1741,36 @@
         <v>3</v>
       </c>
       <c r="K13" s="19" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="L13" s="16" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="M13" s="16" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A14" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="B14" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="C14" s="16" t="s">
+        <v>107</v>
+      </c>
+      <c r="D14" s="16" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A14" s="15" t="s">
-        <v>109</v>
-      </c>
-      <c r="B14" s="15" t="s">
-        <v>67</v>
-      </c>
-      <c r="C14" s="16" t="s">
-        <v>110</v>
-      </c>
-      <c r="D14" s="16" t="s">
-        <v>111</v>
-      </c>
       <c r="E14" s="27" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="F14" s="15" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="G14" s="15" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="H14" s="17">
         <v>46223</v>
@@ -1779,36 +1783,36 @@
         <v>3</v>
       </c>
       <c r="K14" s="19" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="L14" s="16" t="s">
+        <v>110</v>
+      </c>
+      <c r="M14" s="16" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A15" s="12" t="s">
+        <v>112</v>
+      </c>
+      <c r="B15" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="C15" s="21" t="s">
         <v>113</v>
       </c>
-      <c r="M14" s="16" t="s">
+      <c r="D15" s="21" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A15" s="12" t="s">
+      <c r="E15" s="21" t="s">
         <v>115</v>
       </c>
-      <c r="B15" s="12" t="s">
-        <v>67</v>
-      </c>
-      <c r="C15" s="21" t="s">
+      <c r="F15" s="12" t="s">
         <v>116</v>
       </c>
-      <c r="D15" s="21" t="s">
+      <c r="G15" s="12" t="s">
         <v>117</v>
-      </c>
-      <c r="E15" s="21" t="s">
-        <v>118</v>
-      </c>
-      <c r="F15" s="12" t="s">
-        <v>119</v>
-      </c>
-      <c r="G15" s="12" t="s">
-        <v>120</v>
       </c>
       <c r="H15" s="22">
         <v>46226</v>
@@ -1821,36 +1825,36 @@
         <v>1</v>
       </c>
       <c r="K15" s="10" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="L15" s="21" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="M15" s="21" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A16" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="B16" s="15" t="s">
+        <v>120</v>
+      </c>
+      <c r="C16" s="16" t="s">
+        <v>81</v>
+      </c>
+      <c r="D16" s="16" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A16" s="15" t="s">
-        <v>122</v>
-      </c>
-      <c r="B16" s="15" t="s">
-        <v>123</v>
-      </c>
-      <c r="C16" s="16" t="s">
-        <v>83</v>
-      </c>
-      <c r="D16" s="16" t="s">
-        <v>124</v>
-      </c>
       <c r="E16" s="16" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="F16" s="15" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G16" s="15" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="H16" s="17">
         <v>46227</v>
@@ -1863,36 +1867,36 @@
         <v>3</v>
       </c>
       <c r="K16" s="19" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="L16" s="16" t="s">
+        <v>122</v>
+      </c>
+      <c r="M16" s="16" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A17" s="15" t="s">
+        <v>124</v>
+      </c>
+      <c r="B17" s="15" t="s">
+        <v>120</v>
+      </c>
+      <c r="C17" s="16" t="s">
+        <v>81</v>
+      </c>
+      <c r="D17" s="16" t="s">
         <v>125</v>
       </c>
-      <c r="M16" s="16" t="s">
+      <c r="E17" s="16" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A17" s="15" t="s">
-        <v>127</v>
-      </c>
-      <c r="B17" s="15" t="s">
-        <v>123</v>
-      </c>
-      <c r="C17" s="16" t="s">
-        <v>83</v>
-      </c>
-      <c r="D17" s="16" t="s">
-        <v>128</v>
-      </c>
-      <c r="E17" s="16" t="s">
-        <v>129</v>
-      </c>
       <c r="F17" s="15" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G17" s="15" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="H17" s="17">
         <v>46230</v>
@@ -1905,36 +1909,36 @@
         <v>2</v>
       </c>
       <c r="K17" s="19" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="L17" s="16" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="M17" s="16" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" s="15" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C18" s="16" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="D18" s="16" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="E18" s="16" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="F18" s="15" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="G18" s="15" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="H18" s="17">
         <v>46227</v>
@@ -1947,36 +1951,36 @@
         <v>3</v>
       </c>
       <c r="K18" s="19" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="L18" s="16" t="s">
+        <v>130</v>
+      </c>
+      <c r="M18" s="16" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A19" s="15" t="s">
+        <v>132</v>
+      </c>
+      <c r="B19" s="15" t="s">
+        <v>120</v>
+      </c>
+      <c r="C19" s="16" t="s">
+        <v>97</v>
+      </c>
+      <c r="D19" s="16" t="s">
         <v>133</v>
       </c>
-      <c r="M18" s="16" t="s">
+      <c r="E19" s="16" t="s">
+        <v>104</v>
+      </c>
+      <c r="F19" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="G19" s="15" t="s">
         <v>134</v>
-      </c>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A19" s="15" t="s">
-        <v>135</v>
-      </c>
-      <c r="B19" s="15" t="s">
-        <v>123</v>
-      </c>
-      <c r="C19" s="16" t="s">
-        <v>100</v>
-      </c>
-      <c r="D19" s="16" t="s">
-        <v>136</v>
-      </c>
-      <c r="E19" s="16" t="s">
-        <v>107</v>
-      </c>
-      <c r="F19" s="15" t="s">
-        <v>71</v>
-      </c>
-      <c r="G19" s="15" t="s">
-        <v>137</v>
       </c>
       <c r="H19" s="17">
         <v>46231</v>
@@ -1989,36 +1993,36 @@
         <v>3</v>
       </c>
       <c r="K19" s="19" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="L19" s="16" t="s">
+        <v>135</v>
+      </c>
+      <c r="M19" s="16" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A20" s="15" t="s">
+        <v>137</v>
+      </c>
+      <c r="B20" s="15" t="s">
+        <v>120</v>
+      </c>
+      <c r="C20" s="16" t="s">
+        <v>97</v>
+      </c>
+      <c r="D20" s="16" t="s">
         <v>138</v>
       </c>
-      <c r="M19" s="16" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A20" s="15" t="s">
-        <v>140</v>
-      </c>
-      <c r="B20" s="15" t="s">
-        <v>123</v>
-      </c>
-      <c r="C20" s="16" t="s">
-        <v>100</v>
-      </c>
-      <c r="D20" s="16" t="s">
-        <v>141</v>
-      </c>
       <c r="E20" s="16" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="F20" s="15" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="G20" s="15" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="H20" s="17">
         <v>46227</v>
@@ -2031,36 +2035,36 @@
         <v>3</v>
       </c>
       <c r="K20" s="19" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="L20" s="16" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="M20" s="16" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" s="15" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B21" s="15" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C21" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="D21" s="16" t="s">
+        <v>141</v>
+      </c>
+      <c r="E21" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="D21" s="16" t="s">
-        <v>144</v>
-      </c>
-      <c r="E21" s="16" t="s">
-        <v>70</v>
-      </c>
       <c r="F21" s="15" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="G21" s="15" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="H21" s="17">
         <v>46227</v>
@@ -2073,36 +2077,36 @@
         <v>2</v>
       </c>
       <c r="K21" s="19" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="L21" s="16" t="s">
+        <v>142</v>
+      </c>
+      <c r="M21" s="16" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A22" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="B22" s="15" t="s">
+        <v>120</v>
+      </c>
+      <c r="C22" s="16" t="s">
+        <v>107</v>
+      </c>
+      <c r="D22" s="16" t="s">
         <v>145</v>
       </c>
-      <c r="M21" s="16" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A22" s="15" t="s">
-        <v>147</v>
-      </c>
-      <c r="B22" s="15" t="s">
-        <v>123</v>
-      </c>
-      <c r="C22" s="16" t="s">
-        <v>110</v>
-      </c>
-      <c r="D22" s="16" t="s">
-        <v>148</v>
-      </c>
       <c r="E22" s="20" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="F22" s="15" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G22" s="15" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="H22" s="17">
         <v>46231</v>
@@ -2115,36 +2119,36 @@
         <v>3</v>
       </c>
       <c r="K22" s="19" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="L22" s="16" t="s">
+        <v>146</v>
+      </c>
+      <c r="M22" s="16" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A23" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="B23" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="C23" s="21" t="s">
         <v>149</v>
       </c>
-      <c r="M22" s="16" t="s">
+      <c r="D23" s="21" t="s">
         <v>150</v>
       </c>
-    </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A23" s="12" t="s">
+      <c r="E23" s="21" t="s">
+        <v>115</v>
+      </c>
+      <c r="F23" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="G23" s="12" t="s">
         <v>151</v>
-      </c>
-      <c r="B23" s="12" t="s">
-        <v>123</v>
-      </c>
-      <c r="C23" s="21" t="s">
-        <v>152</v>
-      </c>
-      <c r="D23" s="21" t="s">
-        <v>153</v>
-      </c>
-      <c r="E23" s="21" t="s">
-        <v>118</v>
-      </c>
-      <c r="F23" s="12" t="s">
-        <v>119</v>
-      </c>
-      <c r="G23" s="12" t="s">
-        <v>154</v>
       </c>
       <c r="H23" s="22">
         <v>46233</v>
@@ -2157,36 +2161,36 @@
         <v>1</v>
       </c>
       <c r="K23" s="10" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="L23" s="21" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="M23" s="21" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A24" s="15" t="s">
+        <v>153</v>
+      </c>
+      <c r="B24" s="15" t="s">
+        <v>154</v>
+      </c>
+      <c r="C24" s="16" t="s">
+        <v>97</v>
+      </c>
+      <c r="D24" s="16" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A24" s="15" t="s">
+      <c r="E24" s="16" t="s">
         <v>156</v>
       </c>
-      <c r="B24" s="15" t="s">
-        <v>157</v>
-      </c>
-      <c r="C24" s="16" t="s">
-        <v>100</v>
-      </c>
-      <c r="D24" s="16" t="s">
-        <v>158</v>
-      </c>
-      <c r="E24" s="16" t="s">
-        <v>159</v>
-      </c>
       <c r="F24" s="15" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="G24" s="15" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="H24" s="17">
         <v>46234</v>
@@ -2199,36 +2203,36 @@
         <v>2</v>
       </c>
       <c r="K24" s="19" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="L24" s="16" t="s">
+        <v>157</v>
+      </c>
+      <c r="M24" s="16" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A25" s="15" t="s">
+        <v>159</v>
+      </c>
+      <c r="B25" s="15" t="s">
+        <v>154</v>
+      </c>
+      <c r="C25" s="16" t="s">
+        <v>97</v>
+      </c>
+      <c r="D25" s="16" t="s">
         <v>160</v>
       </c>
-      <c r="M24" s="16" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A25" s="15" t="s">
-        <v>162</v>
-      </c>
-      <c r="B25" s="15" t="s">
-        <v>157</v>
-      </c>
-      <c r="C25" s="16" t="s">
-        <v>100</v>
-      </c>
-      <c r="D25" s="16" t="s">
-        <v>163</v>
-      </c>
       <c r="E25" s="16" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="F25" s="15" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G25" s="15" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="H25" s="17">
         <v>46236</v>
@@ -2241,36 +2245,36 @@
         <v>2</v>
       </c>
       <c r="K25" s="19" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="L25" s="16" t="s">
+        <v>161</v>
+      </c>
+      <c r="M25" s="16" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A26" s="15" t="s">
+        <v>163</v>
+      </c>
+      <c r="B26" s="15" t="s">
+        <v>154</v>
+      </c>
+      <c r="C26" s="16" t="s">
+        <v>97</v>
+      </c>
+      <c r="D26" s="16" t="s">
         <v>164</v>
       </c>
-      <c r="M25" s="16" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A26" s="15" t="s">
-        <v>166</v>
-      </c>
-      <c r="B26" s="15" t="s">
-        <v>157</v>
-      </c>
-      <c r="C26" s="16" t="s">
-        <v>100</v>
-      </c>
-      <c r="D26" s="16" t="s">
-        <v>167</v>
-      </c>
       <c r="E26" s="16" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="F26" s="15" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="G26" s="15" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="H26" s="17">
         <v>46234</v>
@@ -2283,36 +2287,36 @@
         <v>2</v>
       </c>
       <c r="K26" s="19" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="L26" s="16" t="s">
+        <v>165</v>
+      </c>
+      <c r="M26" s="16" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A27" s="15" t="s">
+        <v>167</v>
+      </c>
+      <c r="B27" s="15" t="s">
+        <v>154</v>
+      </c>
+      <c r="C27" s="16" t="s">
         <v>168</v>
       </c>
-      <c r="M26" s="16" t="s">
+      <c r="D27" s="16" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A27" s="15" t="s">
-        <v>170</v>
-      </c>
-      <c r="B27" s="15" t="s">
-        <v>157</v>
-      </c>
-      <c r="C27" s="16" t="s">
-        <v>171</v>
-      </c>
-      <c r="D27" s="16" t="s">
-        <v>172</v>
-      </c>
       <c r="E27" s="16" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="F27" s="15" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="G27" s="15" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="H27" s="17">
         <v>46238</v>
@@ -2325,36 +2329,36 @@
         <v>2</v>
       </c>
       <c r="K27" s="19" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="L27" s="16" t="s">
+        <v>170</v>
+      </c>
+      <c r="M27" s="16" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A28" s="15" t="s">
+        <v>172</v>
+      </c>
+      <c r="B28" s="15" t="s">
+        <v>154</v>
+      </c>
+      <c r="C28" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="D28" s="16" t="s">
         <v>173</v>
       </c>
-      <c r="M27" s="16" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A28" s="15" t="s">
-        <v>175</v>
-      </c>
-      <c r="B28" s="15" t="s">
-        <v>157</v>
-      </c>
-      <c r="C28" s="16" t="s">
+      <c r="E28" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="D28" s="16" t="s">
-        <v>176</v>
-      </c>
-      <c r="E28" s="16" t="s">
-        <v>70</v>
-      </c>
       <c r="F28" s="15" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="G28" s="15" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="H28" s="17">
         <v>46234</v>
@@ -2367,36 +2371,36 @@
         <v>2</v>
       </c>
       <c r="K28" s="19" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="L28" s="16" t="s">
+        <v>174</v>
+      </c>
+      <c r="M28" s="16" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A29" s="15" t="s">
+        <v>176</v>
+      </c>
+      <c r="B29" s="15" t="s">
+        <v>154</v>
+      </c>
+      <c r="C29" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="D29" s="16" t="s">
         <v>177</v>
       </c>
-      <c r="M28" s="16" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A29" s="15" t="s">
-        <v>179</v>
-      </c>
-      <c r="B29" s="15" t="s">
-        <v>157</v>
-      </c>
-      <c r="C29" s="16" t="s">
+      <c r="E29" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="D29" s="16" t="s">
-        <v>180</v>
-      </c>
-      <c r="E29" s="16" t="s">
-        <v>70</v>
-      </c>
       <c r="F29" s="15" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G29" s="15" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="H29" s="17">
         <v>46239</v>
@@ -2409,36 +2413,36 @@
         <v>2</v>
       </c>
       <c r="K29" s="19" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="L29" s="16" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="M29" s="16" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" s="15" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="B30" s="15" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="C30" s="16" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="D30" s="16" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="E30" s="20" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="F30" s="15" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G30" s="15" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="H30" s="17">
         <v>46236</v>
@@ -2451,36 +2455,36 @@
         <v>3</v>
       </c>
       <c r="K30" s="19" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="L30" s="16" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="M30" s="16" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A31" s="15" t="s">
+        <v>182</v>
+      </c>
+      <c r="B31" s="15" t="s">
+        <v>154</v>
+      </c>
+      <c r="C31" s="16" t="s">
+        <v>107</v>
+      </c>
+      <c r="D31" s="16" t="s">
+        <v>183</v>
+      </c>
+      <c r="E31" s="20" t="s">
+        <v>109</v>
+      </c>
+      <c r="F31" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="G31" s="15" t="s">
         <v>184</v>
-      </c>
-    </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A31" s="15" t="s">
-        <v>185</v>
-      </c>
-      <c r="B31" s="15" t="s">
-        <v>157</v>
-      </c>
-      <c r="C31" s="16" t="s">
-        <v>110</v>
-      </c>
-      <c r="D31" s="16" t="s">
-        <v>186</v>
-      </c>
-      <c r="E31" s="20" t="s">
-        <v>112</v>
-      </c>
-      <c r="F31" s="15" t="s">
-        <v>78</v>
-      </c>
-      <c r="G31" s="15" t="s">
-        <v>187</v>
       </c>
       <c r="H31" s="17">
         <v>46239</v>
@@ -2493,36 +2497,36 @@
         <v>1</v>
       </c>
       <c r="K31" s="19" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="L31" s="16" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="M31" s="16" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A32" s="12" t="s">
+        <v>186</v>
+      </c>
+      <c r="B32" s="12" t="s">
+        <v>154</v>
+      </c>
+      <c r="C32" s="21" t="s">
+        <v>187</v>
+      </c>
+      <c r="D32" s="21" t="s">
         <v>188</v>
       </c>
-    </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A32" s="12" t="s">
+      <c r="E32" s="21" t="s">
+        <v>115</v>
+      </c>
+      <c r="F32" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="G32" s="12" t="s">
         <v>189</v>
-      </c>
-      <c r="B32" s="12" t="s">
-        <v>157</v>
-      </c>
-      <c r="C32" s="21" t="s">
-        <v>190</v>
-      </c>
-      <c r="D32" s="21" t="s">
-        <v>191</v>
-      </c>
-      <c r="E32" s="21" t="s">
-        <v>118</v>
-      </c>
-      <c r="F32" s="12" t="s">
-        <v>119</v>
-      </c>
-      <c r="G32" s="12" t="s">
-        <v>192</v>
       </c>
       <c r="H32" s="22">
         <v>46240</v>
@@ -2535,58 +2539,57 @@
         <v>1</v>
       </c>
       <c r="K32" s="10" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="L32" s="21" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="M32" s="21" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="35" spans="3:4" x14ac:dyDescent="0.35">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="35" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C35" s="24" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="36" spans="3:4" x14ac:dyDescent="0.35">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="36" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C36" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="D36" s="25">
         <f>COUNTA(A7:A32)</f>
         <v>26</v>
       </c>
     </row>
-    <row r="37" spans="3:4" x14ac:dyDescent="0.35">
+    <row r="37" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C37" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="D37" s="25">
-        <f>COUNTIF(K7:K32, "Completado")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="3:4" x14ac:dyDescent="0.35">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="38" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C38" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="D38" s="25">
         <f>COUNTIF(K7:K32, "In Progress")</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="39" spans="3:4" x14ac:dyDescent="0.35">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="39" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C39" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="D39" s="26">
         <f>(COUNTIF(K7:K32, "Completado") + COUNTIF(K7:K32, "In Progress")*0.5)/COUNTA(A7:A32)</f>
-        <v>5.7692307692307696E-2</v>
+        <v>3.8461538461538464E-2</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A6:M28" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A6:M32" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: actualizar Colab con propuesta de data simple
</commit_message>
<xml_diff>
--- a/Team72_Energi_AI_Sprint_Planner.xlsx
+++ b/Team72_Energi_AI_Sprint_Planner.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Desktop\Google Drive sincronizar\NoCountry Hackaton ONE\Project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Zuleyca Soto\Desktop\ONE ALURA\hackathon\github\G9-LATAM-Team-72-EnergiAI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{049E31A3-01A6-4845-BAF0-EA9B0BBC94FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B860C335-8B0A-486D-A10C-A08353B25D7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Resumen y Equipo" sheetId="1" r:id="rId1"/>
@@ -666,59 +666,59 @@
       <sz val="9"/>
       <color rgb="FF7F7F7F"/>
       <name val="Calibri"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="16"/>
       <color rgb="FF1F4E78"/>
       <name val="Calibri"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="11"/>
       <color rgb="FF595959"/>
       <name val="Calibri"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
       <color rgb="FF1F4E78"/>
       <name val="Calibri"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="11"/>
       <name val="Calibri"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF1F4E78"/>
       <name val="Calibri"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="10">
@@ -1150,34 +1150,34 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C29"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="44.7109375" customWidth="1"/>
+    <col min="1" max="1" width="44.7265625" customWidth="1"/>
     <col min="2" max="2" width="25" customWidth="1"/>
     <col min="3" max="3" width="75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="5" t="s">
         <v>4</v>
       </c>
@@ -1188,7 +1188,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="6" t="s">
         <v>7</v>
       </c>
@@ -1200,7 +1200,7 @@
         <v>Ir a Resumen</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="s">
         <v>8</v>
       </c>
@@ -1212,12 +1212,12 @@
         <v>Ir a Cronograma</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" s="5" t="s">
         <v>11</v>
       </c>
@@ -1228,7 +1228,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" s="6" t="s">
         <v>14</v>
       </c>
@@ -1239,7 +1239,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" s="6" t="s">
         <v>17</v>
       </c>
@@ -1250,7 +1250,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" s="6" t="s">
         <v>20</v>
       </c>
@@ -1261,7 +1261,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" s="6" t="s">
         <v>22</v>
       </c>
@@ -1272,7 +1272,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" s="6" t="s">
         <v>197</v>
       </c>
@@ -1283,7 +1283,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" s="6" t="s">
         <v>26</v>
       </c>
@@ -1294,7 +1294,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" s="6" t="s">
         <v>28</v>
       </c>
@@ -1305,7 +1305,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" s="6" t="s">
         <v>30</v>
       </c>
@@ -1316,12 +1316,12 @@
         <v>32</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="4" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" s="5" t="s">
         <v>34</v>
       </c>
@@ -1332,7 +1332,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26" s="10" t="s">
         <v>37</v>
       </c>
@@ -1343,7 +1343,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27" s="11" t="s">
         <v>40</v>
       </c>
@@ -1354,7 +1354,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28" s="12" t="s">
         <v>43</v>
       </c>
@@ -1365,7 +1365,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A29" s="13" t="s">
         <v>46</v>
       </c>
@@ -1385,37 +1385,37 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:M39"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="77" customWidth="1"/>
     <col min="2" max="2" width="11" customWidth="1"/>
     <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="64.7109375" customWidth="1"/>
+    <col min="4" max="4" width="64.7265625" customWidth="1"/>
     <col min="5" max="5" width="21" customWidth="1"/>
     <col min="6" max="6" width="15" customWidth="1"/>
     <col min="7" max="7" width="21" customWidth="1"/>
     <col min="8" max="9" width="13" customWidth="1"/>
     <col min="10" max="11" width="12" customWidth="1"/>
-    <col min="12" max="12" width="29.5703125" customWidth="1"/>
-    <col min="13" max="13" width="69.85546875" customWidth="1"/>
+    <col min="12" max="12" width="29.54296875" customWidth="1"/>
+    <col min="13" max="13" width="69.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A3" s="2" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="14" t="s">
         <v>51</v>
       </c>
@@ -1456,7 +1456,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" s="15" t="s">
         <v>64</v>
       </c>
@@ -1498,7 +1498,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A8" s="15" t="s">
         <v>74</v>
       </c>
@@ -1540,7 +1540,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A9" s="15" t="s">
         <v>80</v>
       </c>
@@ -1582,7 +1582,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A10" s="15" t="s">
         <v>85</v>
       </c>
@@ -1615,7 +1615,7 @@
         <v>2</v>
       </c>
       <c r="K10" s="19" t="s">
-        <v>77</v>
+        <v>200</v>
       </c>
       <c r="L10" s="16" t="s">
         <v>88</v>
@@ -1624,7 +1624,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11" s="15" t="s">
         <v>90</v>
       </c>
@@ -1666,7 +1666,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A12" s="15" t="s">
         <v>96</v>
       </c>
@@ -1708,7 +1708,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A13" s="15" t="s">
         <v>102</v>
       </c>
@@ -1750,7 +1750,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A14" s="15" t="s">
         <v>106</v>
       </c>
@@ -1783,7 +1783,7 @@
         <v>3</v>
       </c>
       <c r="K14" s="19" t="s">
-        <v>77</v>
+        <v>200</v>
       </c>
       <c r="L14" s="16" t="s">
         <v>110</v>
@@ -1792,7 +1792,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A15" s="12" t="s">
         <v>112</v>
       </c>
@@ -1834,7 +1834,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A16" s="15" t="s">
         <v>119</v>
       </c>
@@ -1876,7 +1876,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A17" s="15" t="s">
         <v>124</v>
       </c>
@@ -1918,7 +1918,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A18" s="15" t="s">
         <v>128</v>
       </c>
@@ -1960,7 +1960,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A19" s="15" t="s">
         <v>132</v>
       </c>
@@ -2002,7 +2002,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A20" s="15" t="s">
         <v>137</v>
       </c>
@@ -2044,7 +2044,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A21" s="15" t="s">
         <v>140</v>
       </c>
@@ -2086,7 +2086,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A22" s="15" t="s">
         <v>144</v>
       </c>
@@ -2128,7 +2128,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A23" s="12" t="s">
         <v>148</v>
       </c>
@@ -2170,7 +2170,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A24" s="15" t="s">
         <v>153</v>
       </c>
@@ -2212,7 +2212,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A25" s="15" t="s">
         <v>159</v>
       </c>
@@ -2254,7 +2254,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A26" s="15" t="s">
         <v>163</v>
       </c>
@@ -2296,7 +2296,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A27" s="15" t="s">
         <v>167</v>
       </c>
@@ -2338,7 +2338,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A28" s="15" t="s">
         <v>172</v>
       </c>
@@ -2380,7 +2380,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A29" s="15" t="s">
         <v>176</v>
       </c>
@@ -2422,7 +2422,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A30" s="15" t="s">
         <v>179</v>
       </c>
@@ -2464,7 +2464,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A31" s="15" t="s">
         <v>182</v>
       </c>
@@ -2506,7 +2506,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A32" s="12" t="s">
         <v>186</v>
       </c>
@@ -2548,12 +2548,12 @@
         <v>190</v>
       </c>
     </row>
-    <row r="35" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C35" s="24" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="36" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C36" t="s">
         <v>192</v>
       </c>
@@ -2562,7 +2562,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="37" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C37" t="s">
         <v>193</v>
       </c>
@@ -2570,7 +2570,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="38" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C38" t="s">
         <v>194</v>
       </c>
@@ -2579,7 +2579,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="39" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C39" t="s">
         <v>195</v>
       </c>

</xml_diff>